<commit_message>
v03: unify bank codes (BNxx) with X011 clearing, rebuild bank/POS controls, audit
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Mazandasht_v03/00_Master.xlsx
+++ b/Mazandasht_v03/00_Master.xlsx
@@ -54,7 +54,7 @@
     <definedName name="OpTbl">Op!$A$10:$S$33</definedName>
     <definedName name="ParamTbl">Par!$A$10:$E$21</definedName>
     <definedName name="ProductTbl">Prd!$B$10:$D$29</definedName>
-    <definedName name="ListBankOps">List!$S$10:$S$25</definedName>
+    <definedName name="ListBankOps">List!$S$10:$S$29</definedName>
     <definedName name="ListOtherScalesLabel">List!$T$10:$T$29</definedName>
     <definedName name="ListBankNames">List!$U$10:$U$19</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Home'!$A$1:$J$46</definedName>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="U8" s="150" t="inlineStr">
         <is>
-          <t>بانک عامل (نام)</t>
+          <t>بانک عامل (کد و نام)</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4187,7 @@
       </c>
       <c r="U10" s="152" t="inlineStr">
         <is>
-          <t>BANK01 – صادرات ۹۰۰۹ — جاری اصلی</t>
+          <t>BN01 – صادرات ۹۰۰۹ — جاری اصلی</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="U11" s="152" t="inlineStr">
         <is>
-          <t>BANK02 – صادرات ۲۰۰۶ — پوز باسکول</t>
+          <t>BN02 – صادرات ۲۰۰۶ — پوز باسکول</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="U12" s="152" t="inlineStr">
         <is>
-          <t>BANK03 – ملت</t>
+          <t>BN03 – ملت</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4460,7 @@
       </c>
       <c r="U13" s="152" t="inlineStr">
         <is>
-          <t>BANK04 – کشاورزی</t>
+          <t>BN04 – کشاورزی</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4519,7 @@
       </c>
       <c r="U14" s="152" t="inlineStr">
         <is>
-          <t>BANK05 – سپه</t>
+          <t>BN05 – سپه</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="U15" s="152" t="inlineStr">
         <is>
-          <t>BANK06 – مهر ایران</t>
+          <t>BN06 – مهر ایران</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="U16" s="152" t="inlineStr">
         <is>
-          <t>BANK07 – تجارت</t>
+          <t>BN07 – تجارت</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="U17" s="152" t="inlineStr">
         <is>
-          <t>BANK08 – پاسارگاد</t>
+          <t>BN08 – پاسارگاد</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="U18" s="152" t="inlineStr">
         <is>
-          <t>BANK09 – رفاه</t>
+          <t>BN09 – رفاه</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4754,7 @@
       </c>
       <c r="U19" s="152" t="inlineStr">
         <is>
-          <t>BANK10 – قرض‌الحسنه</t>
+          <t>BN10 – قرض‌الحسنه</t>
         </is>
       </c>
     </row>
@@ -4957,6 +4957,11 @@
       <c r="P26" s="47" t="n"/>
       <c r="Q26" s="47" t="n"/>
       <c r="R26" s="47" t="n"/>
+      <c r="S26" s="152" t="inlineStr">
+        <is>
+          <t>تسویه دریافت (واسط)</t>
+        </is>
+      </c>
       <c r="T26" s="152" t="inlineStr">
         <is>
           <t>BD017 – (بدون نام)</t>
@@ -4982,6 +4987,11 @@
       <c r="P27" s="47" t="n"/>
       <c r="Q27" s="47" t="n"/>
       <c r="R27" s="47" t="n"/>
+      <c r="S27" s="152" t="inlineStr">
+        <is>
+          <t>تسویه پرداخت (واسط)</t>
+        </is>
+      </c>
       <c r="T27" s="152" t="inlineStr">
         <is>
           <t>BD018 – (بدون نام)</t>
@@ -5534,7 +5544,7 @@
       </c>
       <c r="K15" s="155" t="inlineStr">
         <is>
-          <t>X002</t>
+          <t>X011</t>
         </is>
       </c>
     </row>
@@ -5821,6 +5831,26 @@
       <c r="D23" s="110" t="n"/>
       <c r="E23" s="110" t="n"/>
       <c r="F23" s="110" t="n"/>
+      <c r="H23" s="154" t="inlineStr">
+        <is>
+          <t>تسویه دریافت (واسط)</t>
+        </is>
+      </c>
+      <c r="I23" s="155" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="J23" s="155" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="K23" s="155" t="inlineStr">
+        <is>
+          <t>X011</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="92" t="inlineStr">
@@ -5845,6 +5875,26 @@
           <t>شیت منبع</t>
         </is>
       </c>
+      <c r="H24" s="154" t="inlineStr">
+        <is>
+          <t>تسویه پرداخت (واسط)</t>
+        </is>
+      </c>
+      <c r="I24" s="155" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="J24" s="155" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="K24" s="155" t="inlineStr">
+        <is>
+          <t>X011</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="21" customHeight="1">
       <c r="A25" s="93" t="inlineStr">
@@ -6077,6 +6127,8 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
+    <row r="38"/>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
@@ -6479,6 +6531,7 @@
       <c r="I5" s="112" t="n"/>
       <c r="J5" s="113" t="n"/>
     </row>
+    <row r="6"/>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
@@ -6691,6 +6744,8 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
+    <row r="25"/>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
@@ -6740,6 +6795,7 @@
       <c r="I29" s="112" t="n"/>
       <c r="J29" s="113" t="n"/>
     </row>
+    <row r="30"/>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
@@ -6789,6 +6845,7 @@
       <c r="I34" s="112" t="n"/>
       <c r="J34" s="113" t="n"/>
     </row>
+    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
@@ -6812,7 +6869,7 @@
     <row r="37" ht="96" customHeight="1">
       <c r="B37" s="101" t="inlineStr">
         <is>
-          <t>کدها ثابت‌اند و هرگز عوض نمی‌شوند؛ فقط عنوان‌ها آزادند. پیشوند کد، گروه حساب را نشان می‌دهد: C باغدار (مثلاً C001)، SL بارفروش (SL001)، S فروشنده سبد و تأمین‌کننده (S001)، E کارمند (E001)، X حساب معین داخلی (X001)، BD باسکول دیگران (BD001)، F دارایی ثابت (F001)، L وام (L001) و CAP سرمایه (CAP001). عملیات با OP شروع می‌شود (OP01)، سبد با BK (BK01)، محصول با PB (PB01)، پارامتر با P (P01) و بانک با BANK (BANK01).</t>
+          <t>کدها ثابت‌اند و هرگز عوض نمی‌شوند؛ فقط عنوان‌ها آزادند. پیشوند کد، گروه حساب را نشان می‌دهد: C باغدار (مثلاً C001)، SL بارفروش (SL001)، S فروشنده سبد و تأمین‌کننده (S001)، E کارمند (E001)، X حساب معین داخلی (X001)، BD باسکول دیگران (BD001)، F دارایی ثابت (F001)، L وام (L001) و CAP سرمایه (CAP001). عملیات با OP شروع می‌شود (OP01)، سبد با BK (BK01)، محصول با PB (PB01)، پارامتر با P (P01) و بانک با BANK (BN01).</t>
         </is>
       </c>
     </row>
@@ -6838,6 +6895,7 @@
       <c r="I39" s="112" t="n"/>
       <c r="J39" s="113" t="n"/>
     </row>
+    <row r="40"/>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
@@ -6894,6 +6952,7 @@
       <c r="I45" s="112" t="n"/>
       <c r="J45" s="113" t="n"/>
     </row>
+    <row r="46"/>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="11" t="inlineStr">
         <is>
@@ -6943,6 +7002,7 @@
       <c r="I50" s="112" t="n"/>
       <c r="J50" s="113" t="n"/>
     </row>
+    <row r="51"/>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="11" t="inlineStr">
         <is>
@@ -7020,6 +7080,7 @@
       <c r="I59" s="112" t="n"/>
       <c r="J59" s="113" t="n"/>
     </row>
+    <row r="60"/>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="11" t="inlineStr">
         <is>
@@ -7076,6 +7137,7 @@
       <c r="I65" s="112" t="n"/>
       <c r="J65" s="113" t="n"/>
     </row>
+    <row r="66"/>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="11" t="inlineStr">
         <is>
@@ -7125,6 +7187,7 @@
       <c r="I70" s="112" t="n"/>
       <c r="J70" s="113" t="n"/>
     </row>
+    <row r="71"/>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="11" t="inlineStr">
         <is>
@@ -7148,7 +7211,7 @@
     <row r="73" ht="81" customHeight="1">
       <c r="B73" s="101" t="inlineStr">
         <is>
-          <t>شیت Products نام محصول، دسته (نوع مرکبات)، واحد و سبد پیش‌فرض را نگه می‌دارد. در باسکول با انتخاب محصول، دسته و سبد پیش‌فرض خودکار می‌آید. شیت Banks ده حساب بانکی شرکت را با کد ثابت نگه می‌دارد. کد BANK02 مخصوص «صادرات ۲۰۰۶» و پوز باسکول است؛ عملیات انعام، فروش بار و درآمد پوز همه به همین حساب اشاره می‌کنند. اگر روزی پوز را به حساب دیگری وصل کردید، فقط ستون «بانک پوز» در شیت Ops را عوض کنید.</t>
+          <t>شیت Products نام محصول، دسته (نوع مرکبات)، واحد و سبد پیش‌فرض را نگه می‌دارد. در باسکول با انتخاب محصول، دسته و سبد پیش‌فرض خودکار می‌آید. شیت Banks ده حساب بانکی شرکت را با کد ثابت نگه می‌دارد. کد BN02 مخصوص «صادرات ۲۰۰۶» و پوز باسکول است؛ عملیات انعام، فروش بار و درآمد پوز همه به همین حساب اشاره می‌کنند. اگر روزی پوز را به حساب دیگری وصل کردید، فقط ستون «بانک پوز» در شیت Ops را عوض کنید.</t>
         </is>
       </c>
     </row>
@@ -7174,6 +7237,7 @@
       <c r="I75" s="112" t="n"/>
       <c r="J75" s="113" t="n"/>
     </row>
+    <row r="76"/>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="11" t="inlineStr">
         <is>
@@ -7211,7 +7275,7 @@
     <row r="80" ht="66" customHeight="1">
       <c r="B80" s="101" t="inlineStr">
         <is>
-          <t>سبد جدید: در شیت Baskets ردیف خالی بعدی (BK09) را پر کنید؛ وزن تار را حتماً بنویسید. محصول جدید: در Products ردیف بعدی را پر کنید و سبد پیش‌فرض را انتخاب کنید. بانک جدید: فقط تا BANK10 جا داریم؛ اگر بیشتر شد، شیت Banks و فایل بانک را گسترش دهید.</t>
+          <t>سبد جدید: در شیت Baskets ردیف خالی بعدی (BK09) را پر کنید؛ وزن تار را حتماً بنویسید. محصول جدید: در Products ردیف بعدی را پر کنید و سبد پیش‌فرض را انتخاب کنید. بانک جدید: فقط تا BN10 جا داریم؛ اگر بیشتر شد، شیت Banks و فایل بانک را گسترش دهید.</t>
         </is>
       </c>
     </row>
@@ -7230,6 +7294,7 @@
       <c r="I81" s="112" t="n"/>
       <c r="J81" s="113" t="n"/>
     </row>
+    <row r="82"/>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="11" t="inlineStr">
         <is>
@@ -7279,6 +7344,7 @@
       <c r="I86" s="112" t="n"/>
       <c r="J86" s="113" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
         <is>
@@ -7335,6 +7401,7 @@
       <c r="I92" s="112" t="n"/>
       <c r="J92" s="113" t="n"/>
     </row>
+    <row r="93"/>
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="11" t="inlineStr">
         <is>
@@ -7384,6 +7451,7 @@
       <c r="I97" s="112" t="n"/>
       <c r="J97" s="113" t="n"/>
     </row>
+    <row r="98"/>
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="11" t="inlineStr">
         <is>
@@ -7433,6 +7501,7 @@
       <c r="I102" s="112" t="n"/>
       <c r="J102" s="113" t="n"/>
     </row>
+    <row r="103"/>
     <row r="104" ht="30" customHeight="1">
       <c r="A104" s="11" t="inlineStr">
         <is>
@@ -7482,6 +7551,7 @@
       <c r="I107" s="112" t="n"/>
       <c r="J107" s="113" t="n"/>
     </row>
+    <row r="108"/>
     <row r="109" ht="30" customHeight="1">
       <c r="A109" s="11" t="inlineStr">
         <is>
@@ -7795,6 +7865,7 @@
       <c r="I5" s="110" t="n"/>
       <c r="J5" s="110" t="n"/>
     </row>
+    <row r="6"/>
     <row r="7" ht="26.25" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
         <is>
@@ -8035,6 +8106,7 @@
       <c r="I17" s="112" t="n"/>
       <c r="J17" s="113" t="n"/>
     </row>
+    <row r="18"/>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
@@ -14335,7 +14407,7 @@
       </c>
       <c r="D91" s="65" t="inlineStr">
         <is>
-          <t>حساب واسط عملیات</t>
+          <t>حساب واسط بانک و پز (در راه)</t>
         </is>
       </c>
       <c r="E91" s="65" t="n"/>
@@ -20116,7 +20188,7 @@
       </c>
       <c r="M11" s="59" t="inlineStr">
         <is>
-          <t>BANK02</t>
+          <t>BN02</t>
         </is>
       </c>
       <c r="N11" s="59" t="inlineStr">
@@ -20209,7 +20281,7 @@
       </c>
       <c r="M12" s="59" t="inlineStr">
         <is>
-          <t>BANK02</t>
+          <t>BN02</t>
         </is>
       </c>
       <c r="N12" s="59" t="inlineStr">
@@ -20367,7 +20439,7 @@
       </c>
       <c r="I14" s="59" t="inlineStr">
         <is>
-          <t>BANK02</t>
+          <t>BN02</t>
         </is>
       </c>
       <c r="J14" s="59" t="inlineStr">
@@ -20557,7 +20629,7 @@
       </c>
       <c r="M16" s="59" t="inlineStr">
         <is>
-          <t>BANK02</t>
+          <t>BN02</t>
         </is>
       </c>
       <c r="N16" s="59" t="inlineStr">
@@ -21156,7 +21228,7 @@
       </c>
       <c r="M23" s="59" t="inlineStr">
         <is>
-          <t>BANK02</t>
+          <t>BN02</t>
         </is>
       </c>
       <c r="N23" s="59" t="inlineStr">
@@ -23467,7 +23539,7 @@
       </c>
       <c r="D8" s="42" t="inlineStr">
         <is>
-          <t>شماره حساب</t>
+          <t>کد حساب معین</t>
         </is>
       </c>
       <c r="E8" s="42" t="inlineStr">
@@ -23504,7 +23576,7 @@
       </c>
       <c r="D9" s="43" t="inlineStr">
         <is>
-          <t>Account No.</t>
+          <t>Ledger</t>
         </is>
       </c>
       <c r="E9" s="43" t="inlineStr">
@@ -23526,7 +23598,7 @@
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="44" t="inlineStr">
         <is>
-          <t>BANK01</t>
+          <t>BN01</t>
         </is>
       </c>
       <c r="B10" s="45" t="inlineStr">
@@ -23557,7 +23629,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="44" t="inlineStr">
         <is>
-          <t>BANK02</t>
+          <t>BN02</t>
         </is>
       </c>
       <c r="B11" s="45" t="inlineStr">
@@ -23588,7 +23660,7 @@
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="44" t="inlineStr">
         <is>
-          <t>BANK03</t>
+          <t>BN03</t>
         </is>
       </c>
       <c r="B12" s="45" t="inlineStr">
@@ -23615,7 +23687,7 @@
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="44" t="inlineStr">
         <is>
-          <t>BANK04</t>
+          <t>BN04</t>
         </is>
       </c>
       <c r="B13" s="45" t="inlineStr">
@@ -23642,7 +23714,7 @@
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="44" t="inlineStr">
         <is>
-          <t>BANK05</t>
+          <t>BN05</t>
         </is>
       </c>
       <c r="B14" s="45" t="inlineStr">
@@ -23669,7 +23741,7 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="44" t="inlineStr">
         <is>
-          <t>BANK06</t>
+          <t>BN06</t>
         </is>
       </c>
       <c r="B15" s="45" t="inlineStr">
@@ -23696,7 +23768,7 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="44" t="inlineStr">
         <is>
-          <t>BANK07</t>
+          <t>BN07</t>
         </is>
       </c>
       <c r="B16" s="45" t="inlineStr">
@@ -23723,7 +23795,7 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="44" t="inlineStr">
         <is>
-          <t>BANK08</t>
+          <t>BN08</t>
         </is>
       </c>
       <c r="B17" s="45" t="inlineStr">
@@ -23750,7 +23822,7 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="44" t="inlineStr">
         <is>
-          <t>BANK09</t>
+          <t>BN09</t>
         </is>
       </c>
       <c r="B18" s="45" t="inlineStr">
@@ -23777,7 +23849,7 @@
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="44" t="inlineStr">
         <is>
-          <t>BANK10</t>
+          <t>BN10</t>
         </is>
       </c>
       <c r="B19" s="45" t="inlineStr">

</xml_diff>